<commit_message>
docs(examples): complete conditional-formatting and document-formatting into full quartets
Both showcases previously shipped without their sh CLI generator. Add it so each
is a full quartet (md walkthrough of the CLI + sh CLI twin + py SDK twin + product),
the sh being the canonical form the md explains and the gate that proves every key
is a real CLI-accepted canonical key under `set -e`.

Also note in document-formatting.md that the bare `sectPr=present` toggle is
intentionally not demonstrated: it is an internal dump->batch round-trip marker
(get-invisible, single-valued), settable only for fidelity, never an interactive
edit -- mirroring the auto-assigned table `id` skip note in tables-nested.

Products regenerated from the final scripts.
</commit_message>
<xml_diff>
--- a/examples/excel/conditional-formatting.xlsx
+++ b/examples/excel/conditional-formatting.xlsx
@@ -3,12 +3,12 @@
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="rId1"/>
-    <x:sheet name="Text" sheetId="2" r:id="Rcba0102082da4466"/>
-    <x:sheet name="TopBottom" sheetId="3" r:id="R3d57eb50f90942dd"/>
-    <x:sheet name="DataBars" sheetId="4" r:id="R961b6054f0d54455"/>
-    <x:sheet name="ColorScales" sheetId="5" r:id="R4540262f19594aea"/>
-    <x:sheet name="IconSets" sheetId="6" r:id="R53777feaea764ac6"/>
-    <x:sheet name="FormulaEtc" sheetId="7" r:id="Rc0c4359ffb5342ed"/>
+    <x:sheet name="Text" sheetId="2" r:id="R27e7e081ad87409b"/>
+    <x:sheet name="TopBottom" sheetId="3" r:id="Ra0cf2f5af5554cee"/>
+    <x:sheet name="DataBars" sheetId="4" r:id="R1242ca48bbc14336"/>
+    <x:sheet name="ColorScales" sheetId="5" r:id="R9eb819191b6243da"/>
+    <x:sheet name="IconSets" sheetId="6" r:id="R1cc9806bc19147be"/>
+    <x:sheet name="FormulaEtc" sheetId="7" r:id="Rb3b89e43d6594cd8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -194,6 +194,115 @@
 </x:styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="44546A"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="E7E6E6"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4472C4"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="ED7D31"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="A5A5A5"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="FFC000"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="5B9BD5"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="70AD47"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0563C1"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="954F72"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="6350" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+        </a:ln>
+        <a:ln w="12700" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+        </a:ln>
+        <a:ln w="19050" cap="flat">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData>
@@ -514,7 +623,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{DFF7D76A-4269-49B0-AB8D-CF92AE6F0D28}</x14:id>
+          <x14:id>{0DFB3B2A-D3B2-404A-B40C-9B93736B2ACA}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -523,7 +632,7 @@
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{DFF7D76A-4269-49B0-AB8D-CF92AE6F0D28}">
+          <x14:cfRule type="dataBar" id="{0DFB3B2A-D3B2-404A-B40C-9B93736B2ACA}">
             <x14:dataBar minLength="0" maxLength="100" axisPosition="middle">
               <x14:cfvo type="autoMin"/>
               <x14:cfvo type="autoMax"/>

</xml_diff>